<commit_message>
Aggiornamento menu.xlsx via backend
</commit_message>
<xml_diff>
--- a/menu.xlsx
+++ b/menu.xlsx
@@ -1,50 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Python\Projects\Dati Mensa\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37FCCFE4-A016-4738-808F-470E136FD985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_56BDB0300675BEFF8C4516E5730504BEB6C424A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="menù estate 2026" sheetId="1" r:id="rId1"/>
+    <sheet name="menu autunno 2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="Excel_BuiltIn_Print_Area" localSheetId="0">#N/A</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'menu autunno 2026'!$A$1:$G$40</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="136">
-  <si>
-    <t>MENU LEONARDO CASCINA COSTA  2026 – ESTATE    DAL 22/06/26</t>
-  </si>
-  <si>
-    <t>MENU ESTATE LEONARDO 2026</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="143">
+  <si>
+    <t>MENU LEONARDO CASCINA COSTA 2026 - AUTUNNO DAL 05/10/26</t>
+  </si>
+  <si>
+    <t>MENU AUTUNNO LEONARDO 2026</t>
   </si>
   <si>
     <t>SETTIMANA 1</t>
@@ -62,398 +47,419 @@
     <t>LUNEDI</t>
   </si>
   <si>
-    <t>PASTA AL POMODORO FRESCO E RUCOLA</t>
+    <t>GNOCCHI AL PESTO</t>
+  </si>
+  <si>
+    <t>PASTA ALLA CARRETTIERA</t>
+  </si>
+  <si>
+    <t>PASTA ALLA PIEMONTESE</t>
+  </si>
+  <si>
+    <t>PASTA ALLA PUTTANESCA</t>
+  </si>
+  <si>
+    <t>PASTA CON BROCCOLI E SALSICCIA</t>
+  </si>
+  <si>
+    <t>PASTA AL RADICCHIO</t>
+  </si>
+  <si>
+    <t>PASTA SALSICCIA E PEPERONI</t>
+  </si>
+  <si>
+    <t>PASTA AL SALMONE AFFUMICATO</t>
+  </si>
+  <si>
+    <t>ZUPPA DI CANNELLINI</t>
+  </si>
+  <si>
+    <t>ZUPPA DI CECI</t>
+  </si>
+  <si>
+    <t>MINESTRONE DI VERDURA</t>
+  </si>
+  <si>
+    <t>ZUPPA DI VERDURA</t>
+  </si>
+  <si>
+    <t>FILETTO DI PERSICO AGLI AGRUMI</t>
+  </si>
+  <si>
+    <t>SPEZZATINO DI TACCHINO CON PISELLI</t>
+  </si>
+  <si>
+    <t>COSCIA DI POLLO ARROSTO</t>
+  </si>
+  <si>
+    <t>BOCCONCINI DI TACCHINO CON FUNGHI E VERDURE</t>
+  </si>
+  <si>
+    <t>COSCIA DI POLLO PICCANTE</t>
+  </si>
+  <si>
+    <t>TORTA DI RICOTTA E SPINACI</t>
+  </si>
+  <si>
+    <t>SOFFICINO AL FORMAGGIO</t>
+  </si>
+  <si>
+    <t>FILETTO DI MERLUZZO IMPANATO</t>
+  </si>
+  <si>
+    <t>FILETTO DI MERLUZZO ALLO ZENZERO</t>
+  </si>
+  <si>
+    <t>FILETTO DI NASELLO AL PEPE E CURCUMA</t>
+  </si>
+  <si>
+    <t>FARINATA DI CECI ZUCCHINE E ROSMARINO</t>
+  </si>
+  <si>
+    <t>CAVOLFIORI</t>
+  </si>
+  <si>
+    <t>MIX DI VERDURE</t>
+  </si>
+  <si>
+    <t>CAROTE</t>
+  </si>
+  <si>
+    <t>MARTEDI</t>
+  </si>
+  <si>
+    <t>PASTA ALL'AMATRICIANA</t>
+  </si>
+  <si>
+    <t>PASTA ALLE CIME DI RAPA</t>
+  </si>
+  <si>
+    <t>RISOTTO ALLO STRACCHINO E ZUCCHINE</t>
+  </si>
+  <si>
+    <t>RISOTTO ALLA MILANESE</t>
+  </si>
+  <si>
+    <t>PASTA AL POMODORO E TONNO</t>
+  </si>
+  <si>
+    <t>PASTA AI CARCIOFI</t>
+  </si>
+  <si>
+    <t>PASTA AL POMODORO ROSMARINO E PATATE</t>
+  </si>
+  <si>
+    <t>PASTA AL POMODORO E BASILICO</t>
+  </si>
+  <si>
+    <t>MINESTRA DI VERDURA</t>
+  </si>
+  <si>
+    <t>ZUPPA DI SEDANO</t>
+  </si>
+  <si>
+    <t>ZUPPA DI PORRI</t>
+  </si>
+  <si>
+    <t>CASSOEUOLA</t>
+  </si>
+  <si>
+    <t>KEBAB</t>
+  </si>
+  <si>
+    <t>ARISTA CON VERDURINE ALL’AGRO</t>
+  </si>
+  <si>
+    <t>ROAST BEEF CON RUCOLA</t>
+  </si>
+  <si>
+    <t>GATEAUX DI PATATE AL FORMAGGIO</t>
+  </si>
+  <si>
+    <t>FRITTATA CON VERDURE</t>
+  </si>
+  <si>
+    <t>FILETTO DI MERLUZZO IN BAGNETTO</t>
+  </si>
+  <si>
+    <t>TORTA RUSTICA ALLE ZUCCHINE</t>
+  </si>
+  <si>
+    <t>INSALATA DI TONNO FAGIOLINI E OLIVE</t>
+  </si>
+  <si>
+    <t>FILETTO DI PERSICO PREZZEMOLATO</t>
+  </si>
+  <si>
+    <t>TORTINO ARRAGANATO</t>
+  </si>
+  <si>
+    <t>FETTUCCINE DI TOTANO CON PISELLI IN COCCIO</t>
+  </si>
+  <si>
+    <t>LENTICCHIE IN UMIDO</t>
+  </si>
+  <si>
+    <t>FAGIOLI CANNELLINI STUFATI</t>
+  </si>
+  <si>
+    <t>FAGIOLI BORLOTTI STUFATI</t>
+  </si>
+  <si>
+    <t>MERCOLEDI</t>
+  </si>
+  <si>
+    <t>RISOTTO ALLA ZUCCA</t>
+  </si>
+  <si>
+    <t>RISOTTO AI FUNGHI</t>
+  </si>
+  <si>
+    <t>PASTA ALL'ARRABBIATA</t>
+  </si>
+  <si>
+    <t>PASTA AI 4 FORMAGGI</t>
+  </si>
+  <si>
+    <t>PASTA AL RAGU' DI VERDURE</t>
+  </si>
+  <si>
+    <t>PASTA AL POMODORO E CAPPERI</t>
+  </si>
+  <si>
+    <t>GNOCCHI ALLA SORRENTINA</t>
   </si>
   <si>
     <t>PASTA AL TONNO</t>
   </si>
   <si>
-    <t>INSALATA DI PASTA AL POMODORO FRESCO  E ORIGANO</t>
-  </si>
-  <si>
-    <t>PASTA ALLA PUTTANESCA</t>
-  </si>
-  <si>
-    <t>PASTA AI PEPERONI</t>
-  </si>
-  <si>
-    <t>MISTO CEREALI QUARTIROLO E VERDURE</t>
-  </si>
-  <si>
-    <t>PASTA ALLE CIME DI RAPA</t>
-  </si>
-  <si>
-    <t>INSALATA DI FARRO VEGETARIANA</t>
-  </si>
-  <si>
-    <t>MINESTRONE  DI VERDURA</t>
-  </si>
-  <si>
-    <t>ZUPPA DI VERDURA</t>
-  </si>
-  <si>
-    <t>CREMA PARMANTIER</t>
-  </si>
-  <si>
-    <t>INSALATA DI TONNO FAGIOLINI ,PATATE E OLIVE</t>
-  </si>
-  <si>
-    <t>BOCCONCINI DI TACCHINO AL CURRY</t>
-  </si>
-  <si>
-    <t>COSCIA DI POLLO ARROSTO</t>
-  </si>
-  <si>
-    <t>WURSTELL E CRAUTI</t>
-  </si>
-  <si>
-    <t>COSCIA DI POLLO ALLA DIAVOLA</t>
-  </si>
-  <si>
-    <t>TORTA PASQUALINA</t>
-  </si>
-  <si>
-    <t>SOFFICINO AL FORMAGGIO</t>
-  </si>
-  <si>
-    <t>FILETTO DI MERLUZZO PANATO</t>
-  </si>
-  <si>
-    <t>FILETTO DI DI MERLUZZO ALLA GRENOBLESE</t>
-  </si>
-  <si>
-    <t>INSALATA DI TONNO FAGIOLI E PATATE</t>
-  </si>
-  <si>
-    <t>SPEZZATINO VEGANO CON FAVE</t>
-  </si>
-  <si>
-    <t>CAVOLFIORI</t>
-  </si>
-  <si>
-    <t>MIX DI VERDURE</t>
-  </si>
-  <si>
-    <t>MISTO LEGUMI</t>
-  </si>
-  <si>
-    <t>MARTEDÌ</t>
-  </si>
-  <si>
-    <t>PASTA ALL'AMATRICIANA</t>
-  </si>
-  <si>
-    <t>PASTA  ALLA NORMA</t>
-  </si>
-  <si>
-    <t>INSALATA DI RISO VEGETARIANA</t>
-  </si>
-  <si>
-    <t>PASTA AI BROCCOLI</t>
-  </si>
-  <si>
-    <t>INSALATA DI PASTA AI CARCIOFI E OLIVE</t>
-  </si>
-  <si>
-    <t>PASTA AL PESTO</t>
-  </si>
-  <si>
-    <t>PASTA AL GAZPACHO</t>
-  </si>
-  <si>
-    <t>PASTA AL SALMONE</t>
-  </si>
-  <si>
-    <t>ZUPPA DI PORRI</t>
-  </si>
-  <si>
-    <t>MINESTRA DI SEDANO</t>
-  </si>
-  <si>
-    <t>MINESTRA DI VERDURA</t>
-  </si>
-  <si>
-    <t>VELLUTATA DI SEDANO</t>
-  </si>
-  <si>
-    <t>KEBAB</t>
-  </si>
-  <si>
-    <t>ARISTA DI MAIALE AL TIMO</t>
-  </si>
-  <si>
-    <t>LONZA ALL'  ALLORO</t>
-  </si>
-  <si>
-    <t>FRITTATA CON VERDURE</t>
-  </si>
-  <si>
-    <t>CAPONATINA   AGRODOLCE IN COCCIO (PIATTO VEGANO)</t>
-  </si>
-  <si>
-    <t>TACCHINO FUME' CON LATTUGA  E OLIVE</t>
-  </si>
-  <si>
-    <t>TORTINO DI PATATE AL ROSMARINO</t>
-  </si>
-  <si>
-    <t>VITELLONE TONNATO</t>
-  </si>
-  <si>
-    <t>FILETTO DI MERLUZZO AL SALMORIGLIO</t>
-  </si>
-  <si>
-    <t>FILETTO DI SCORFANO AL BAGNETTO DI VERDURE</t>
-  </si>
-  <si>
-    <t>COCCIO DI CANNELLINI  E COZZE</t>
-  </si>
-  <si>
-    <t>FILETTO DI PERSICO ALLA CURCUMA</t>
+    <t>MINESTRA DI PORRI</t>
+  </si>
+  <si>
+    <t>MINESTRA DI ZUCCHINE</t>
+  </si>
+  <si>
+    <t>VELLUTATA DI VERDURA</t>
+  </si>
+  <si>
+    <t>MINESTRA DI CAROTE</t>
+  </si>
+  <si>
+    <t>LOMBO DI MAIALE ARROSTO</t>
+  </si>
+  <si>
+    <t>LONZA ALL'ALLORO</t>
+  </si>
+  <si>
+    <t>BRASATO DI VITELLONE</t>
+  </si>
+  <si>
+    <t>OMELETTE CON FRIARIELLI</t>
+  </si>
+  <si>
+    <t>OMELETTE FORMAGGIO</t>
+  </si>
+  <si>
+    <t>SPEZZATINO VEGANO CON FAVE SPEZIATO AL GINGER</t>
+  </si>
+  <si>
+    <t>PROVOLONE AL FORNO CON POMODORO</t>
+  </si>
+  <si>
+    <t>ARISTA AI CARCIOFI</t>
+  </si>
+  <si>
+    <t>FILETTO DI MERLUZZO IN GUAZZETTO</t>
+  </si>
+  <si>
+    <t>FILETTO DI NASELLO IN UMIDO</t>
+  </si>
+  <si>
+    <t>FILETTO DI SALMONE AL VAPORE</t>
+  </si>
+  <si>
+    <t>FILETTO DI NASELLO AL SALMORIGLIO</t>
+  </si>
+  <si>
+    <t>PATATE AL FORNO</t>
+  </si>
+  <si>
+    <t>POLENTA</t>
   </si>
   <si>
     <t>FINOCCHI</t>
   </si>
   <si>
-    <t>MERCOLEDÌ</t>
-  </si>
-  <si>
-    <t>PASTA AL POMODORO E RICOTTA</t>
-  </si>
-  <si>
-    <t>RISO PILAFF CURCUMA E VERDURE</t>
-  </si>
-  <si>
-    <t>PASTA AL PESTO DI RUCOLA</t>
-  </si>
-  <si>
-    <t>INSALATA DI RISO</t>
-  </si>
-  <si>
-    <t>INSALATA DI RISO ALLA MEDITERRANEA</t>
-  </si>
-  <si>
-    <t>PASTA ALL' ARRABBIATA</t>
-  </si>
-  <si>
-    <t>PASTA AL POMODORO E CAPPERI</t>
-  </si>
-  <si>
-    <t>PASTA  AL POMODORO E BASILICO</t>
-  </si>
-  <si>
-    <t>MINESTRA DI ZUCCHINE</t>
-  </si>
-  <si>
-    <t>MINESTRA DI CAROTE</t>
-  </si>
-  <si>
-    <t>VELLUTATA DI PORRI</t>
-  </si>
-  <si>
-    <t>ZUPPA  DI CANNELLINI</t>
-  </si>
-  <si>
-    <t>FESA DI TACCHINO ARROSTO</t>
-  </si>
-  <si>
-    <t>SCALOPPA GRATINATA</t>
+    <t>GIOVEDI</t>
+  </si>
+  <si>
+    <t>LINGUINE ALL'ARRABBIATA</t>
+  </si>
+  <si>
+    <t>SPAGHETTI ALLA BOLOGNESE</t>
+  </si>
+  <si>
+    <t>PASTA AL POMODORO E VERDURE</t>
+  </si>
+  <si>
+    <t>LASAGNA</t>
+  </si>
+  <si>
+    <t>LINGUINE ALLO SCOGLIO</t>
+  </si>
+  <si>
+    <t>SPAGHETTI ALL'AGLIONE</t>
+  </si>
+  <si>
+    <t>PASTA SPECK E FUNGHI</t>
+  </si>
+  <si>
+    <t>PASTA ALLA PIZZAIOLA</t>
+  </si>
+  <si>
+    <t>ZUPPA DI CAROTE</t>
+  </si>
+  <si>
+    <t>ZUPPA ALLA CONTADINA</t>
+  </si>
+  <si>
+    <t>CREMA DI ZUCCA</t>
+  </si>
+  <si>
+    <t>MINESTRA ALLA CONTADINA</t>
+  </si>
+  <si>
+    <t>INSALATA DI MARE</t>
+  </si>
+  <si>
+    <t>SFORMATO DI ZUCCA</t>
+  </si>
+  <si>
+    <t>SCALOPPA DI MAIALE GRATINATA AGLI AROMI</t>
+  </si>
+  <si>
+    <t>COTOLETTA DI TACCHINO</t>
+  </si>
+  <si>
+    <t>COCCIO DI BROCCOLI STUFATI, OLIVE ED E.V.O. CON CROSTONE</t>
   </si>
   <si>
     <t>ROAST BEEF</t>
   </si>
   <si>
-    <t>ARISTA DI MAIALE AI FUNGHI</t>
-  </si>
-  <si>
-    <t>HUMMUS DI LEGUMI ,MELANZANE E MENTA</t>
-  </si>
-  <si>
-    <t>FILETTO DI PERSICO MARINATO</t>
-  </si>
-  <si>
-    <t>OMELETTE AL FORMAGGIO</t>
-  </si>
-  <si>
-    <t>SFORMATO RUSTICO AI PEPERONI</t>
-  </si>
-  <si>
-    <t>INSALATA DI MARE</t>
-  </si>
-  <si>
-    <t>COCCIO DI ZUCCHINE E UOVA STRAPAZZATE</t>
-  </si>
-  <si>
-    <t>FILETTO DI NASELLO  IN UMIDO</t>
-  </si>
-  <si>
-    <t>FILETTO DI  SCORFANO PREZZEMOLATO</t>
-  </si>
-  <si>
-    <t>CAROTE</t>
+    <t>FILETTO DI SCORFANO ALLA PAPRIKA</t>
+  </si>
+  <si>
+    <t>FILETTO DI MERLUZZO ALLE OLIVE</t>
+  </si>
+  <si>
+    <t>FESA DI TACCHINO COTTA AL VAPORE</t>
+  </si>
+  <si>
+    <t>ZUPPETTA DI PESCE IN COCCIO</t>
+  </si>
+  <si>
+    <t>HUMMUS DI CECI CON CROSTONE</t>
+  </si>
+  <si>
+    <t>CURRY DI VERDURE IN COCCIO</t>
   </si>
   <si>
     <t>FAGIOLINI</t>
   </si>
   <si>
-    <t>GIOVEDÌ</t>
-  </si>
-  <si>
-    <t>RAVIOLI ALLA SORRENTINA</t>
-  </si>
-  <si>
-    <t>INSALATA DI PASTA ALLA ZUCCA E ROSMARINO</t>
-  </si>
-  <si>
-    <t>PASTA ALLA PIZZAIOLA</t>
+    <t>CAVOLINI DI BRUXELLES</t>
+  </si>
+  <si>
+    <t>VENERDI</t>
   </si>
   <si>
     <t>PASTA ALLA PORTOFINO</t>
   </si>
   <si>
-    <t>PASTA AL POMODORO PATATE E ROSMARINO</t>
-  </si>
-  <si>
-    <t>PASTA SPECK E PISELLI</t>
-  </si>
-  <si>
-    <t>RAVIOLI  ALLA BOLOGNESE</t>
-  </si>
-  <si>
-    <t>PASTA AL PESTATO DI ZUCCHINE</t>
-  </si>
-  <si>
-    <t>MINESTRA ALLA CONTADINA</t>
-  </si>
-  <si>
-    <t>ZUPPA DI FAGIOLI CANNELLINI</t>
-  </si>
-  <si>
-    <t>FILETTO DI PERSICO PREZZEMOLATO</t>
-  </si>
-  <si>
-    <t>SFORMATO DI PATATE E ZUCCHINE</t>
-  </si>
-  <si>
-    <t>FESA DI TACCHINO COTTA AL VAPORE CON ZENZERO</t>
-  </si>
-  <si>
-    <t>FESA DI TACCHINO  ALLA MILANESE</t>
-  </si>
-  <si>
-    <t>FRITTATA CON FRIARIELLI</t>
-  </si>
-  <si>
-    <t>INSALATA DI POLLO</t>
-  </si>
-  <si>
-    <t>HUMMUS DI CECI CON CROSTONE</t>
-  </si>
-  <si>
-    <t>FILETTO DI TROTA</t>
-  </si>
-  <si>
-    <t>ROAST-BEEF CON RUCOLA</t>
-  </si>
-  <si>
-    <t>FILETTO DI MERLUZZO  IN GUAZZETTO</t>
-  </si>
-  <si>
-    <t>COCCIO DI LENTICCHIE SENAPE E PATATE</t>
-  </si>
-  <si>
-    <t>CAVOLINI DI BRUXELLES</t>
-  </si>
-  <si>
-    <t>VENERDÌ</t>
-  </si>
-  <si>
-    <t>PASTA ALLA BOLOGNESE</t>
-  </si>
-  <si>
-    <t>PASTA ALLA CARRETTIERA</t>
+    <t>PASTA ALLA PUGLIESE</t>
   </si>
   <si>
     <t>SPAGHETTI AGLIO OLIO E PEPERONCINO</t>
   </si>
   <si>
-    <t>PASTA FREDDA CON VERDURE</t>
-  </si>
-  <si>
-    <t>INSALATA DI PASTA ZUCCHINE E CURCUMA</t>
-  </si>
-  <si>
-    <t>PASTA AL CAVOLO CAPPUCCIO ED EMMENTHAL</t>
-  </si>
-  <si>
-    <t>SPAGHETTI AL POMODORO E ACCIUGA</t>
-  </si>
-  <si>
-    <t>PASTA ALLA PUGLIESE</t>
-  </si>
-  <si>
-    <t>ZUPPA DI FAGIOLI AZUKI</t>
-  </si>
-  <si>
-    <t>PASSATA DI VERDURE</t>
-  </si>
-  <si>
-    <t>PASSATA DI LEGUMI</t>
+    <t>PASTA AL POMODORO E FUNGHI</t>
+  </si>
+  <si>
+    <t>PASTA ALLA PROVOLA FUME'</t>
+  </si>
+  <si>
+    <t>PASTA ALLE VERZE</t>
+  </si>
+  <si>
+    <t>SPAGHETTI ALLA TRAPANESE</t>
+  </si>
+  <si>
+    <t>PASTA ALLE ZUCCHINE</t>
+  </si>
+  <si>
+    <t>ZUPPA DI CAVOLO</t>
   </si>
   <si>
     <t>VELLUTATA DI VERDURE</t>
   </si>
   <si>
-    <t>SCALOPPINA DI MAIALE AGLI AROMI</t>
-  </si>
-  <si>
-    <t>LONZA AL FORNO</t>
+    <t>ZUPPA DI LEGUMI</t>
+  </si>
+  <si>
+    <t>PASSATO DI VERDURA</t>
+  </si>
+  <si>
+    <t>BRACIOLA DI MAIALE IN SALSA MIREPOIX</t>
+  </si>
+  <si>
+    <t>SCALOPPINA ALLA PIZZAIOLA</t>
   </si>
   <si>
     <t>BRACIOLA DI MAIALE AL VINO BIANCO</t>
   </si>
   <si>
-    <t>TACCHINO FUME'  CON RUCOLA</t>
+    <t>TACCHINO FUME' CON RUCOLA</t>
   </si>
   <si>
     <t>FILETTO DI NASELLO GRATINATO</t>
   </si>
   <si>
-    <t>FILETTO DI NASELLO AL LIMONE</t>
-  </si>
-  <si>
-    <t>FILETTO DI  MERLUZZO AGLI AGRUMI</t>
-  </si>
-  <si>
-    <t>INSALATONA CON TONNO</t>
+    <t>FILETTO DI SCORFANO</t>
+  </si>
+  <si>
+    <t>FILETTO DI NASELLO PREZZEMOLATO</t>
+  </si>
+  <si>
+    <t>COCCIO DI PATATE, CREMA DI LATTE GRATINATO</t>
+  </si>
+  <si>
+    <t>BURGHER DI CAROTE E CECI</t>
+  </si>
+  <si>
+    <t>INSALATONA</t>
   </si>
   <si>
     <t>BURGHER DI BROCCOLI</t>
   </si>
   <si>
-    <t>INSALATONA</t>
-  </si>
-  <si>
-    <t>BURGHER VEGETARIANI AI PISELLI E CAROTE</t>
-  </si>
-  <si>
-    <t>LONZA AL LATTE</t>
+    <t>SCALOPPINA DI MAIALE AL BURRO E SALVIA</t>
   </si>
   <si>
     <t>PATATE AL VAPORE</t>
   </si>
   <si>
+    <t>PATATE PREZZEMOLATE</t>
+  </si>
+  <si>
     <t>BIETA ERBETTA</t>
-  </si>
-  <si>
-    <t>PATATE PREZZEMOLATE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -819,21 +825,21 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1262,27 +1268,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G40"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="16.5" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="2" width="13.28515625" style="1" customWidth="1"/>
     <col min="3" max="6" width="50.28515625" style="1" customWidth="1"/>
     <col min="7" max="7" width="8.85546875" style="2" customWidth="1"/>
     <col min="8" max="8" width="50.7109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="2"/>
+    <col min="9" max="10" width="8.85546875" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:6" ht="26.25" customHeight="1">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-    </row>
-    <row r="2" spans="1:6" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+    </row>
+    <row r="2" spans="1:6" ht="26.25" customHeight="1">
       <c r="A2" s="18"/>
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
@@ -1290,12 +1296,12 @@
       <c r="E2" s="18"/>
       <c r="F2" s="18"/>
     </row>
-    <row r="3" spans="1:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:6" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="8.25" customHeight="1"/>
+    <row r="4" spans="1:6" ht="40.5" customHeight="1" thickBot="1">
       <c r="A4" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="20"/>
+      <c r="B4" s="23"/>
       <c r="C4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1309,11 +1315,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="21" t="s">
+    <row r="5" spans="1:6" ht="25.15" customHeight="1">
+      <c r="A5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="22"/>
+      <c r="B5" s="24"/>
       <c r="C5" s="5" t="s">
         <v>7</v>
       </c>
@@ -1327,9 +1333,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="23"/>
-      <c r="B6" s="24"/>
+    <row r="6" spans="1:6" ht="34.5" customHeight="1">
+      <c r="A6" s="25"/>
+      <c r="B6" s="26"/>
       <c r="C6" s="7" t="s">
         <v>11</v>
       </c>
@@ -1343,9 +1349,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="23"/>
-      <c r="B7" s="24"/>
+    <row r="7" spans="1:6" ht="25.15" customHeight="1">
+      <c r="A7" s="25"/>
+      <c r="B7" s="26"/>
       <c r="C7" s="7" t="s">
         <v>15</v>
       </c>
@@ -1356,126 +1362,126 @@
         <v>17</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="23"/>
-      <c r="B8" s="24"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="25.15" customHeight="1">
+      <c r="A8" s="25"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="23"/>
-      <c r="B9" s="24"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="25.15" customHeight="1">
+      <c r="A9" s="25"/>
+      <c r="B9" s="26"/>
       <c r="C9" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F9" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="25.15" customHeight="1">
+      <c r="A10" s="25"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="7" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="23"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="7" t="s">
-        <v>24</v>
-      </c>
       <c r="D10" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="25"/>
-      <c r="B11" s="26"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="25.15" customHeight="1" thickBot="1">
+      <c r="A11" s="27"/>
+      <c r="B11" s="28"/>
       <c r="C11" s="17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E11" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="22"/>
+    </row>
+    <row r="12" spans="1:6" ht="25.15" customHeight="1">
+      <c r="A12" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="24"/>
       <c r="C12" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="23"/>
-      <c r="B13" s="24"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="30.75" customHeight="1">
+      <c r="A13" s="25"/>
+      <c r="B13" s="26"/>
       <c r="C13" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="23"/>
-      <c r="B14" s="24"/>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="30.75" customHeight="1">
+      <c r="A14" s="25"/>
+      <c r="B14" s="26"/>
       <c r="C14" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E14" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F14" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F14" s="8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="23"/>
-      <c r="B15" s="24"/>
+    </row>
+    <row r="15" spans="1:6" ht="32.25" customHeight="1">
+      <c r="A15" s="25"/>
+      <c r="B15" s="26"/>
       <c r="C15" s="7" t="s">
         <v>45</v>
       </c>
@@ -1489,9 +1495,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="23"/>
-      <c r="B16" s="24"/>
+    <row r="16" spans="1:6" ht="32.25" customHeight="1">
+      <c r="A16" s="25"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="7" t="s">
         <v>49</v>
       </c>
@@ -1505,9 +1511,9 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="23"/>
-      <c r="B17" s="24"/>
+    <row r="17" spans="1:7" ht="34.5" customHeight="1">
+      <c r="A17" s="25"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="7" t="s">
         <v>53</v>
       </c>
@@ -1521,372 +1527,372 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="11" customFormat="1" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="25"/>
-      <c r="B18" s="26"/>
+    <row r="18" spans="1:7" s="11" customFormat="1" ht="25.15" customHeight="1" thickBot="1">
+      <c r="A18" s="27"/>
+      <c r="B18" s="28"/>
       <c r="C18" s="17" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>57</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="B19" s="22"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="25.15" customHeight="1">
+      <c r="A19" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="24"/>
       <c r="C19" s="7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="23"/>
-      <c r="B20" s="24"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="25.15" customHeight="1">
+      <c r="A20" s="25"/>
+      <c r="B20" s="26"/>
       <c r="C20" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="23"/>
-      <c r="B21" s="24"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="25.15" customHeight="1">
+      <c r="A21" s="25"/>
+      <c r="B21" s="26"/>
       <c r="C21" s="12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="23"/>
-      <c r="B22" s="24"/>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="26.25" customHeight="1">
+      <c r="A22" s="25"/>
+      <c r="B22" s="26"/>
       <c r="C22" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="23"/>
-      <c r="B23" s="24"/>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="30.75" customHeight="1">
+      <c r="A23" s="25"/>
+      <c r="B23" s="26"/>
       <c r="C23" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="23"/>
-      <c r="B24" s="24"/>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="25.15" customHeight="1">
+      <c r="A24" s="25"/>
+      <c r="B24" s="26"/>
       <c r="C24" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" s="13" customFormat="1" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="25"/>
-      <c r="B25" s="26"/>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" s="13" customFormat="1" ht="25.15" customHeight="1" thickBot="1">
+      <c r="A25" s="27"/>
+      <c r="B25" s="28"/>
       <c r="C25" s="17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="B26" s="22"/>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="25.15" customHeight="1">
+      <c r="A26" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B26" s="24"/>
       <c r="C26" s="5" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G26" s="14"/>
     </row>
-    <row r="27" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="23"/>
-      <c r="B27" s="24"/>
+    <row r="27" spans="1:7" ht="25.15" customHeight="1">
+      <c r="A27" s="25"/>
+      <c r="B27" s="26"/>
       <c r="C27" s="7" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G27" s="14"/>
     </row>
-    <row r="28" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="23"/>
-      <c r="B28" s="24"/>
+    <row r="28" spans="1:7" ht="25.15" customHeight="1">
+      <c r="A28" s="25"/>
+      <c r="B28" s="26"/>
       <c r="C28" s="7" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="G28" s="14"/>
     </row>
-    <row r="29" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="23"/>
-      <c r="B29" s="24"/>
+    <row r="29" spans="1:7" ht="25.15" customHeight="1">
+      <c r="A29" s="25"/>
+      <c r="B29" s="26"/>
       <c r="C29" s="7" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="G29" s="14"/>
     </row>
-    <row r="30" spans="1:7" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="23"/>
-      <c r="B30" s="24"/>
+    <row r="30" spans="1:7" ht="32.450000000000003" customHeight="1">
+      <c r="A30" s="25"/>
+      <c r="B30" s="26"/>
       <c r="C30" s="7" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="G30" s="14"/>
     </row>
-    <row r="31" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="23"/>
-      <c r="B31" s="24"/>
+    <row r="31" spans="1:7" ht="37.5" customHeight="1">
+      <c r="A31" s="25"/>
+      <c r="B31" s="26"/>
       <c r="C31" s="7" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>79</v>
+        <v>111</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="G31" s="14"/>
     </row>
-    <row r="32" spans="1:7" s="15" customFormat="1" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="25"/>
-      <c r="B32" s="26"/>
+    <row r="32" spans="1:7" s="15" customFormat="1" ht="25.15" customHeight="1" thickBot="1">
+      <c r="A32" s="27"/>
+      <c r="B32" s="28"/>
       <c r="C32" s="17" t="s">
-        <v>57</v>
+        <v>113</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>107</v>
+        <v>30</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="G32" s="14"/>
     </row>
-    <row r="33" spans="1:6" ht="30.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="B33" s="22"/>
+    <row r="33" spans="1:6" ht="30.6" customHeight="1">
+      <c r="A33" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="B33" s="24"/>
       <c r="C33" s="5" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="23"/>
-      <c r="B34" s="24"/>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="31.5" customHeight="1">
+      <c r="A34" s="25"/>
+      <c r="B34" s="26"/>
       <c r="C34" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="31.5" customHeight="1">
+      <c r="A35" s="25"/>
+      <c r="B35" s="26"/>
+      <c r="C35" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="25.15" customHeight="1">
+      <c r="A36" s="25"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F36" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="37.5" customHeight="1">
+      <c r="A37" s="25"/>
+      <c r="B37" s="26"/>
+      <c r="C37" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="35.25" customHeight="1">
+      <c r="A38" s="25"/>
+      <c r="B38" s="26"/>
+      <c r="C38" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="25.15" customHeight="1" thickBot="1">
+      <c r="A39" s="27"/>
+      <c r="B39" s="28"/>
+      <c r="C39" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="D39" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="D34" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="E34" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="23"/>
-      <c r="B35" s="24"/>
-      <c r="C35" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="23"/>
-      <c r="B36" s="24"/>
-      <c r="C36" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="E36" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="F36" s="10" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="23"/>
-      <c r="B37" s="24"/>
-      <c r="C37" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="E37" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="F37" s="8" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="23"/>
-      <c r="B38" s="24"/>
-      <c r="C38" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="E38" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="25"/>
-      <c r="B39" s="26"/>
-      <c r="C39" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="D39" s="17" t="s">
-        <v>133</v>
-      </c>
       <c r="E39" s="17" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="27" customHeight="1">
       <c r="A40" s="16"/>
       <c r="B40" s="16"/>
       <c r="C40" s="16"/>
@@ -1906,10 +1912,10 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="54" firstPageNumber="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="54" firstPageNumber="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter alignWithMargins="0">
-    <oddFooter>&amp;C&amp;"Aptos Narrow"&amp;11&amp;K000000&amp;"Calibri"&amp;10 &amp;K000000#Company General Use_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000Company General Use</oddFooter>
+    <oddFooter>&amp;C&amp;"Aptos Narrow"&amp;11&amp;K000000&amp;"Calibri"&amp;10 &amp;K000000#Company General Use_x000D_&amp;1#&amp;"Calibri"&amp;10 &amp;K000000Company General Use</oddFooter>
   </headerFooter>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>